<commit_message>
changed colors and font
</commit_message>
<xml_diff>
--- a/excel files/Table Supp-All columns.xlsx
+++ b/excel files/Table Supp-All columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valentinamelica/R/Best-Practices-Parallelism/excel files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B16EA83-18AE-224A-93D7-07D4F602A89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D358A6A-2E12-B445-8A71-6649C384C6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="980" yWindow="500" windowWidth="27820" windowHeight="17500" xr2:uid="{591C8C7C-A714-0C40-8252-48F48B9A1CF9}"/>
   </bookViews>
@@ -304,26 +304,26 @@
     <t>Determined based on aim of the study, the species/population investigated and the ournal</t>
   </si>
   <si>
-    <t>pertianing free-ranging  wildlife population,  with clear conservation efforts in midn</t>
+    <t>Studies focusing on behavior, cognition or animal welfare in domesticated species or species under human care (including both wild and lab animals). These studies typically investigate how housing, environmental or management conditions influence behavior and/or welfare metrics, and HPA axis activity is used as an indicator.</t>
   </si>
   <si>
-    <t xml:space="preserve">Physiological prosesses, with particular attention (but not exclusive)  to reproduction in wildlife populations, both free ranging or under human care </t>
+    <t>Studies focusing on reproduction, stress physiology, and hormonal regulation. These studies typically include investigating baseline endocrinology for a species, evaluating different assay techniques and validation of hormonal assays, and investigations of biological mechanisms of hormone production or variation. In these studies, hormones are the main object of study rather than a tool to address ecological, welfare, or conservation questions.</t>
   </si>
   <si>
-    <t>pertaining stress response  population/species under human care, domesitcated or maintained in a laboratory setting.</t>
+    <t>Studies conducted on free-ranging wildlife populations with a focus on ecological processes, population dynamics, species interactions or conservation outcomes. Hormonal measures are used to understand responses to environmental variation, anthropogenic disturbance, or ecological pressures, with a clear conservation or ecological framework.</t>
   </si>
   <si>
-    <t>studies investigating immune response in captive animals</t>
+    <t>Studies using animal models to investigate neurological, cognitive, behavioral, or mental health-related processes, typically under controlled experimental conditions. The primary aim is to address biomedical or mechanistic questions relevant to neuroscience or translational research, where the animal functions as a model system. In this category, stress and behavioral measures are not used to evaluate welfare or improve husbandry conditions for the study species.</t>
   </si>
   <si>
-    <t xml:space="preserve">studies investigating neurological and mental health related  processes that may have implication to biomedical research and </t>
+    <t>Studies focusing on animal health, disease, pathology, microbiology or clinical interventions, where physiological stress markers are clearly used in relation to health status, disease processes or treatment outcomes.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -349,6 +349,12 @@
       <i/>
       <sz val="12"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0C64C0"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -468,7 +474,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -825,7 +831,7 @@
     <col min="1" max="1" width="63.83203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="59.33203125" style="2" customWidth="1"/>
     <col min="3" max="3" width="43.33203125" style="8" customWidth="1"/>
-    <col min="4" max="4" width="35.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="90.1640625" style="2" customWidth="1"/>
     <col min="5" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
@@ -868,7 +874,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>5</v>
       </c>
@@ -879,10 +885,10 @@
         <v>64</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A8" s="10"/>
       <c r="B8" s="13"/>
       <c r="C8" s="7" t="s">
@@ -892,34 +898,34 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
       <c r="B9" s="13"/>
       <c r="C9" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A10" s="10"/>
       <c r="B10" s="13"/>
       <c r="C10" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="11"/>
       <c r="B11" s="14"/>
       <c r="C11" s="7" t="s">
         <v>63</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>